<commit_message>
ahora si ultimo cambio
</commit_message>
<xml_diff>
--- a/Pauta/E01Pauta.xlsx
+++ b/Pauta/E01Pauta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub Clones\polla-mundial\Pauta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09941CAB-0568-4713-84D3-C2C25FA276D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D0C29C-EBBF-482C-ACCC-1519C0627458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14655" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{80BA0768-A233-4C15-9128-A9DFED026552}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="59">
   <si>
     <t>Partido 1</t>
   </si>
@@ -391,27 +391,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -431,6 +410,27 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -784,26 +784,24 @@
   <sheetData>
     <row r="2" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="3" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="17"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="11"/>
     </row>
     <row r="4" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="14"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="8"/>
     </row>
     <row r="5" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="6" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="8"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="17"/>
       <c r="H6" s="2" t="str">
         <f>"Gana "&amp;B7</f>
         <v>Gana México</v>
@@ -825,20 +823,20 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="9"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="11"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="14"/>
       <c r="H8" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="10" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="8"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
       <c r="H10" s="2" t="str">
         <f>"Gana "&amp;B11</f>
         <v>Gana Estados Unidos</v>
@@ -860,20 +858,20 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="9"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="11"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="14"/>
       <c r="H12" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="14" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="8"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
       <c r="H14" s="2" t="str">
         <f>"Gana "&amp;B15</f>
         <v>Gana Brasil</v>
@@ -895,20 +893,20 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="9"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="14"/>
       <c r="H16" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="18" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="8"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="17"/>
       <c r="H18" s="2" t="str">
         <f>"Gana "&amp;B19</f>
         <v>Gana Australia</v>
@@ -931,20 +929,20 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B20" s="9"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="11"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="14"/>
       <c r="H20" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="22" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="8"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="17"/>
       <c r="H22" s="2" t="str">
         <f>"Gana "&amp;B23</f>
         <v>Gana Holanda</v>
@@ -966,20 +964,20 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B24" s="9"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="14"/>
       <c r="H24" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="26" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="8"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="17"/>
       <c r="H26" s="2" t="str">
         <f>"Gana "&amp;B27</f>
         <v>Gana Bélgica</v>
@@ -1001,20 +999,20 @@
       </c>
     </row>
     <row r="28" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="9"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="11"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="14"/>
       <c r="H28" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="30" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="8"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="17"/>
       <c r="H30" s="2" t="str">
         <f>"Gana "&amp;B31</f>
         <v>Gana Francia</v>
@@ -1036,20 +1034,20 @@
       </c>
     </row>
     <row r="32" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B32" s="9"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="11"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="14"/>
       <c r="H32" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="34" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C34" s="7"/>
-      <c r="D34" s="8"/>
+      <c r="C34" s="16"/>
+      <c r="D34" s="17"/>
       <c r="H34" s="2" t="str">
         <f>"Gana "&amp;B35</f>
         <v>Gana Argentina</v>
@@ -1071,20 +1069,20 @@
       </c>
     </row>
     <row r="36" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B36" s="9"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="11"/>
+      <c r="B36" s="12"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="14"/>
       <c r="H36" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="38" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C38" s="7"/>
-      <c r="D38" s="8"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="17"/>
       <c r="H38" s="2" t="str">
         <f>"Gana "&amp;B39</f>
         <v>Gana Inglaterra</v>
@@ -1107,20 +1105,20 @@
       </c>
     </row>
     <row r="40" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B40" s="9"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="11"/>
+      <c r="B40" s="12"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="14"/>
       <c r="H40" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="42" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C42" s="7"/>
-      <c r="D42" s="8"/>
+      <c r="C42" s="16"/>
+      <c r="D42" s="17"/>
       <c r="H42" s="2" t="str">
         <f>"Gana "&amp;B43</f>
         <v>Gana México</v>
@@ -1142,20 +1140,20 @@
       </c>
     </row>
     <row r="44" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B44" s="9"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="11"/>
+      <c r="B44" s="12"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="14"/>
       <c r="H44" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="45" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="46" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C46" s="7"/>
-      <c r="D46" s="8"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="17"/>
       <c r="H46" s="2" t="str">
         <f>"Gana "&amp;B47</f>
         <v>Gana Estados Unidos</v>
@@ -1177,20 +1175,20 @@
       </c>
     </row>
     <row r="48" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B48" s="9"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="11"/>
+      <c r="B48" s="12"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="14"/>
       <c r="H48" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="49" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="50" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B50" s="6" t="s">
+      <c r="B50" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C50" s="7"/>
-      <c r="D50" s="8"/>
+      <c r="C50" s="16"/>
+      <c r="D50" s="17"/>
       <c r="H50" s="2" t="str">
         <f>"Gana "&amp;B51</f>
         <v>Gana Holanda</v>
@@ -1212,20 +1210,20 @@
       </c>
     </row>
     <row r="52" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B52" s="9"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="11"/>
+      <c r="B52" s="12"/>
+      <c r="C52" s="13"/>
+      <c r="D52" s="14"/>
       <c r="H52" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="53" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="54" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C54" s="7"/>
-      <c r="D54" s="8"/>
+      <c r="C54" s="16"/>
+      <c r="D54" s="17"/>
       <c r="H54" s="2" t="str">
         <f>"Gana "&amp;B55</f>
         <v>Gana Bélgica</v>
@@ -1247,20 +1245,20 @@
       </c>
     </row>
     <row r="56" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B56" s="9"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="11"/>
+      <c r="B56" s="12"/>
+      <c r="C56" s="13"/>
+      <c r="D56" s="14"/>
       <c r="H56" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="57" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="58" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B58" s="6" t="s">
+      <c r="B58" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C58" s="7"/>
-      <c r="D58" s="8"/>
+      <c r="C58" s="16"/>
+      <c r="D58" s="17"/>
       <c r="H58" s="2" t="str">
         <f>"Gana "&amp;B59</f>
         <v>Gana Argentina</v>
@@ -1283,20 +1281,20 @@
       </c>
     </row>
     <row r="60" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B60" s="9"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="11"/>
+      <c r="B60" s="12"/>
+      <c r="C60" s="13"/>
+      <c r="D60" s="14"/>
       <c r="H60" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="61" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="62" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B62" s="6" t="s">
+      <c r="B62" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C62" s="7"/>
-      <c r="D62" s="8"/>
+      <c r="C62" s="16"/>
+      <c r="D62" s="17"/>
       <c r="H62" s="2" t="str">
         <f>"Gana "&amp;B63</f>
         <v>Gana Noruega</v>
@@ -1318,20 +1316,20 @@
       </c>
     </row>
     <row r="64" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B64" s="9"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="11"/>
+      <c r="B64" s="12"/>
+      <c r="C64" s="13"/>
+      <c r="D64" s="14"/>
       <c r="H64" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="65" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="66" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B66" s="6" t="s">
+      <c r="B66" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="7"/>
-      <c r="D66" s="8"/>
+      <c r="C66" s="16"/>
+      <c r="D66" s="17"/>
       <c r="H66" s="2" t="str">
         <f>"Gana "&amp;B67</f>
         <v>Gana Suiza</v>
@@ -1353,20 +1351,20 @@
       </c>
     </row>
     <row r="68" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B68" s="9"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="11"/>
+      <c r="B68" s="12"/>
+      <c r="C68" s="13"/>
+      <c r="D68" s="14"/>
       <c r="H68" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="69" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="70" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B70" s="6" t="s">
+      <c r="B70" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C70" s="7"/>
-      <c r="D70" s="8"/>
+      <c r="C70" s="16"/>
+      <c r="D70" s="17"/>
       <c r="H70" s="2" t="str">
         <f>"Gana "&amp;B71</f>
         <v>Gana Ecuador</v>
@@ -1388,20 +1386,20 @@
       </c>
     </row>
     <row r="72" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B72" s="9"/>
-      <c r="C72" s="10"/>
-      <c r="D72" s="11"/>
+      <c r="B72" s="12"/>
+      <c r="C72" s="13"/>
+      <c r="D72" s="14"/>
       <c r="H72" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="73" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="74" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B74" s="6" t="s">
+      <c r="B74" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C74" s="7"/>
-      <c r="D74" s="8"/>
+      <c r="C74" s="16"/>
+      <c r="D74" s="17"/>
       <c r="H74" s="2" t="str">
         <f>"Gana "&amp;B75</f>
         <v>Gana Japón</v>
@@ -1423,20 +1421,20 @@
       </c>
     </row>
     <row r="76" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B76" s="9"/>
-      <c r="C76" s="10"/>
-      <c r="D76" s="11"/>
+      <c r="B76" s="12"/>
+      <c r="C76" s="13"/>
+      <c r="D76" s="14"/>
       <c r="H76" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="77" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="78" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B78" s="6" t="s">
+      <c r="B78" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C78" s="7"/>
-      <c r="D78" s="8"/>
+      <c r="C78" s="16"/>
+      <c r="D78" s="17"/>
       <c r="H78" s="2" t="str">
         <f>"Gana "&amp;B79</f>
         <v>Gana Turquía</v>
@@ -1459,20 +1457,20 @@
       </c>
     </row>
     <row r="80" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B80" s="9"/>
-      <c r="C80" s="10"/>
-      <c r="D80" s="11"/>
+      <c r="B80" s="12"/>
+      <c r="C80" s="13"/>
+      <c r="D80" s="14"/>
       <c r="H80" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="81" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="82" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B82" s="6" t="s">
+      <c r="B82" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="C82" s="7"/>
-      <c r="D82" s="8"/>
+      <c r="C82" s="16"/>
+      <c r="D82" s="17"/>
       <c r="H82" s="2" t="str">
         <f>"Gana "&amp;B83</f>
         <v>Gana Paraguay</v>
@@ -1494,20 +1492,20 @@
       </c>
     </row>
     <row r="84" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B84" s="9"/>
-      <c r="C84" s="10"/>
-      <c r="D84" s="11"/>
+      <c r="B84" s="12"/>
+      <c r="C84" s="13"/>
+      <c r="D84" s="14"/>
       <c r="H84" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="85" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="86" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B86" s="6" t="s">
+      <c r="B86" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C86" s="7"/>
-      <c r="D86" s="8"/>
+      <c r="C86" s="16"/>
+      <c r="D86" s="17"/>
       <c r="H86" s="2" t="str">
         <f>"Gana "&amp;B87</f>
         <v>Gana Uruguay</v>
@@ -1529,20 +1527,20 @@
       </c>
     </row>
     <row r="88" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B88" s="9"/>
-      <c r="C88" s="10"/>
-      <c r="D88" s="11"/>
+      <c r="B88" s="12"/>
+      <c r="C88" s="13"/>
+      <c r="D88" s="14"/>
       <c r="H88" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="89" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="90" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B90" s="6" t="s">
+      <c r="B90" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="C90" s="7"/>
-      <c r="D90" s="8"/>
+      <c r="C90" s="16"/>
+      <c r="D90" s="17"/>
       <c r="H90" s="2" t="str">
         <f>"Gana "&amp;B91</f>
         <v>Gana Noruega</v>
@@ -1564,20 +1562,20 @@
       </c>
     </row>
     <row r="92" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B92" s="9"/>
-      <c r="C92" s="10"/>
-      <c r="D92" s="11"/>
+      <c r="B92" s="12"/>
+      <c r="C92" s="13"/>
+      <c r="D92" s="14"/>
       <c r="H92" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="93" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="94" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B94" s="6" t="s">
+      <c r="B94" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C94" s="7"/>
-      <c r="D94" s="8"/>
+      <c r="C94" s="16"/>
+      <c r="D94" s="17"/>
       <c r="H94" s="2" t="str">
         <f>"Gana "&amp;B95</f>
         <v>Gana Egipto</v>
@@ -1599,20 +1597,20 @@
       </c>
     </row>
     <row r="96" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B96" s="9"/>
-      <c r="C96" s="10"/>
-      <c r="D96" s="11"/>
+      <c r="B96" s="12"/>
+      <c r="C96" s="13"/>
+      <c r="D96" s="14"/>
       <c r="H96" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="97" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="98" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B98" s="6" t="s">
+      <c r="B98" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C98" s="7"/>
-      <c r="D98" s="8"/>
+      <c r="C98" s="16"/>
+      <c r="D98" s="17"/>
       <c r="H98" s="2" t="str">
         <f>"Gana "&amp;B99</f>
         <v>Gana Argelia</v>
@@ -1634,20 +1632,20 @@
       </c>
     </row>
     <row r="100" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B100" s="9"/>
-      <c r="C100" s="10"/>
-      <c r="D100" s="11"/>
+      <c r="B100" s="12"/>
+      <c r="C100" s="13"/>
+      <c r="D100" s="14"/>
       <c r="H100" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="101" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="102" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B102" s="6" t="s">
+      <c r="B102" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C102" s="7"/>
-      <c r="D102" s="8"/>
+      <c r="C102" s="16"/>
+      <c r="D102" s="17"/>
       <c r="H102" s="2" t="str">
         <f>"Gana "&amp;B103</f>
         <v>Gana Colombia</v>
@@ -1669,9 +1667,9 @@
       </c>
     </row>
     <row r="104" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B104" s="9"/>
-      <c r="C104" s="10"/>
-      <c r="D104" s="11"/>
+      <c r="B104" s="12"/>
+      <c r="C104" s="13"/>
+      <c r="D104" s="14"/>
       <c r="H104" s="2" t="s">
         <v>1</v>
       </c>
@@ -1679,6 +1677,42 @@
   </sheetData>
   <sheetProtection sheet="1" selectLockedCells="1"/>
   <mergeCells count="52">
+    <mergeCell ref="B78:D78"/>
+    <mergeCell ref="B80:D80"/>
+    <mergeCell ref="B82:D82"/>
+    <mergeCell ref="B84:D84"/>
+    <mergeCell ref="B68:D68"/>
+    <mergeCell ref="B70:D70"/>
+    <mergeCell ref="B72:D72"/>
+    <mergeCell ref="B74:D74"/>
+    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B102:D102"/>
+    <mergeCell ref="B104:D104"/>
+    <mergeCell ref="B86:D86"/>
+    <mergeCell ref="B88:D88"/>
+    <mergeCell ref="B90:D90"/>
+    <mergeCell ref="B92:D92"/>
+    <mergeCell ref="B94:D94"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B96:D96"/>
@@ -1695,42 +1729,6 @@
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B102:D102"/>
-    <mergeCell ref="B104:D104"/>
-    <mergeCell ref="B86:D86"/>
-    <mergeCell ref="B88:D88"/>
-    <mergeCell ref="B90:D90"/>
-    <mergeCell ref="B92:D92"/>
-    <mergeCell ref="B94:D94"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="B66:D66"/>
-    <mergeCell ref="B78:D78"/>
-    <mergeCell ref="B80:D80"/>
-    <mergeCell ref="B82:D82"/>
-    <mergeCell ref="B84:D84"/>
-    <mergeCell ref="B68:D68"/>
-    <mergeCell ref="B70:D70"/>
-    <mergeCell ref="B72:D72"/>
-    <mergeCell ref="B74:D74"/>
-    <mergeCell ref="B76:D76"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B100 B96 B8 B12 B16 B20 B24 B28 B32 B36 B40 B44 B48 B52 B56 B60 B64 B68 B72 B76 B80 B84 B88 B92 B104" xr:uid="{5B958DC4-58BD-46F0-BD6B-4A983C6D99F0}">

</xml_diff>